<commit_message>
Release v2.14.0: document scanner TSA proofs
</commit_message>
<xml_diff>
--- a/app/src/main/assets/methodmesh/odk_templates/documentscanner/example_odk_showcase_document_scan.xlsx
+++ b/app/src/main/assets/methodmesh/odk_templates/documentscanner/example_odk_showcase_document_scan.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R23ea1f67d199406d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rdcf29eb89bdc49a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="Rf4a0e64b925048bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" r:id="R80287f23c4fe457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" r:id="Rbdbcab8f99de4a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" r:id="R71449f47d87949ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -336,15 +336,15 @@
       <x:c r="D2" s="8" t="str">
         <x:v>Capture paper pages and return searchable PDF/OCR outputs</x:v>
       </x:c>
-      <x:c r="E2" s="8" t="str"/>
-      <x:c r="F2" s="8" t="str"/>
-      <x:c r="G2" s="8" t="str"/>
-      <x:c r="H2" s="8" t="str"/>
-      <x:c r="I2" s="8" t="str"/>
-      <x:c r="J2" s="8" t="str"/>
-      <x:c r="K2" s="8" t="str"/>
-      <x:c r="L2" s="8" t="str"/>
-      <x:c r="M2" s="8" t="str"/>
+      <x:c r="E2" s="8"/>
+      <x:c r="F2" s="8"/>
+      <x:c r="G2" s="8"/>
+      <x:c r="H2" s="8"/>
+      <x:c r="I2" s="8"/>
+      <x:c r="J2" s="8"/>
+      <x:c r="K2" s="8"/>
+      <x:c r="L2" s="8"/>
+      <x:c r="M2" s="8"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="8" t="str">
@@ -362,15 +362,15 @@
       <x:c r="E3" s="8" t="str">
         <x:v>field-list</x:v>
       </x:c>
-      <x:c r="F3" s="8" t="str"/>
-      <x:c r="G3" s="8" t="str"/>
-      <x:c r="H3" s="8" t="str"/>
-      <x:c r="I3" s="8" t="str"/>
-      <x:c r="J3" s="8" t="str"/>
-      <x:c r="K3" s="8" t="str"/>
-      <x:c r="L3" s="8" t="str"/>
+      <x:c r="F3" s="8"/>
+      <x:c r="G3" s="8"/>
+      <x:c r="H3" s="8"/>
+      <x:c r="I3" s="8"/>
+      <x:c r="J3" s="8"/>
+      <x:c r="K3" s="8"/>
+      <x:c r="L3" s="8"/>
       <x:c r="M3" s="8" t="str">
-        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='document.scan',input_page_limit='10',input_scanner_mode='full',input_allow_gallery_import='true',input_run_ocr='true',input_return_searchable_pdf='true',input_return_text_file='true',input_payload_mode='FULL',return_mode='flat')</x:v>
+        <x:v>com.example.methodmesh.EXECUTE_METHOD(method_id='document.scan',input_page_limit='10',input_scanner_mode='full',input_allow_gallery_import='true',input_run_ocr='true',input_return_searchable_pdf='true',input_return_text_file='true',input_timestamp_policy='preferred',input_payload_mode='FULL',return_mode='flat')</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -386,15 +386,15 @@
       <x:c r="D4" s="8" t="str">
         <x:v>No undocumented ODK inputs have been invented for this showcase.</x:v>
       </x:c>
-      <x:c r="E4" s="8" t="str"/>
-      <x:c r="F4" s="8" t="str"/>
-      <x:c r="G4" s="8" t="str"/>
-      <x:c r="H4" s="8" t="str"/>
-      <x:c r="I4" s="8" t="str"/>
-      <x:c r="J4" s="8" t="str"/>
-      <x:c r="K4" s="8" t="str"/>
-      <x:c r="L4" s="8" t="str"/>
-      <x:c r="M4" s="8" t="str"/>
+      <x:c r="E4" s="8"/>
+      <x:c r="F4" s="8"/>
+      <x:c r="G4" s="8"/>
+      <x:c r="H4" s="8"/>
+      <x:c r="I4" s="8"/>
+      <x:c r="J4" s="8"/>
+      <x:c r="K4" s="8"/>
+      <x:c r="L4" s="8"/>
+      <x:c r="M4" s="8"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
@@ -412,16 +412,16 @@
       <x:c r="E5" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F5" s="8" t="str"/>
-      <x:c r="G5" s="8" t="str"/>
-      <x:c r="H5" s="8" t="str"/>
-      <x:c r="I5" s="8" t="str"/>
-      <x:c r="J5" s="8" t="str"/>
-      <x:c r="K5" s="8" t="str"/>
+      <x:c r="F5" s="8"/>
+      <x:c r="G5" s="8"/>
+      <x:c r="H5" s="8"/>
+      <x:c r="I5" s="8"/>
+      <x:c r="J5" s="8"/>
+      <x:c r="K5" s="8"/>
       <x:c r="L5" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M5" s="8" t="str"/>
+      <x:c r="M5" s="8"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="8" t="str">
@@ -439,16 +439,16 @@
       <x:c r="E6" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F6" s="8" t="str"/>
-      <x:c r="G6" s="8" t="str"/>
-      <x:c r="H6" s="8" t="str"/>
-      <x:c r="I6" s="8" t="str"/>
-      <x:c r="J6" s="8" t="str"/>
-      <x:c r="K6" s="8" t="str"/>
+      <x:c r="F6" s="8"/>
+      <x:c r="G6" s="8"/>
+      <x:c r="H6" s="8"/>
+      <x:c r="I6" s="8"/>
+      <x:c r="J6" s="8"/>
+      <x:c r="K6" s="8"/>
       <x:c r="L6" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M6" s="8" t="str"/>
+      <x:c r="M6" s="8"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="8" t="str">
@@ -466,16 +466,16 @@
       <x:c r="E7" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F7" s="8" t="str"/>
-      <x:c r="G7" s="8" t="str"/>
-      <x:c r="H7" s="8" t="str"/>
-      <x:c r="I7" s="8" t="str"/>
-      <x:c r="J7" s="8" t="str"/>
-      <x:c r="K7" s="8" t="str"/>
+      <x:c r="F7" s="8"/>
+      <x:c r="G7" s="8"/>
+      <x:c r="H7" s="8"/>
+      <x:c r="I7" s="8"/>
+      <x:c r="J7" s="8"/>
+      <x:c r="K7" s="8"/>
       <x:c r="L7" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M7" s="8" t="str"/>
+      <x:c r="M7" s="8"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="8" t="str">
@@ -493,16 +493,16 @@
       <x:c r="E8" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F8" s="8" t="str"/>
-      <x:c r="G8" s="8" t="str"/>
-      <x:c r="H8" s="8" t="str"/>
-      <x:c r="I8" s="8" t="str"/>
-      <x:c r="J8" s="8" t="str"/>
-      <x:c r="K8" s="8" t="str"/>
+      <x:c r="F8" s="8"/>
+      <x:c r="G8" s="8"/>
+      <x:c r="H8" s="8"/>
+      <x:c r="I8" s="8"/>
+      <x:c r="J8" s="8"/>
+      <x:c r="K8" s="8"/>
       <x:c r="L8" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M8" s="8" t="str"/>
+      <x:c r="M8" s="8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="8" t="str">
@@ -520,16 +520,16 @@
       <x:c r="E9" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F9" s="8" t="str"/>
-      <x:c r="G9" s="8" t="str"/>
-      <x:c r="H9" s="8" t="str"/>
-      <x:c r="I9" s="8" t="str"/>
-      <x:c r="J9" s="8" t="str"/>
-      <x:c r="K9" s="8" t="str"/>
+      <x:c r="F9" s="8"/>
+      <x:c r="G9" s="8"/>
+      <x:c r="H9" s="8"/>
+      <x:c r="I9" s="8"/>
+      <x:c r="J9" s="8"/>
+      <x:c r="K9" s="8"/>
       <x:c r="L9" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M9" s="8" t="str"/>
+      <x:c r="M9" s="8"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="8" t="str">
@@ -547,16 +547,16 @@
       <x:c r="E10" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F10" s="8" t="str"/>
-      <x:c r="G10" s="8" t="str"/>
-      <x:c r="H10" s="8" t="str"/>
-      <x:c r="I10" s="8" t="str"/>
-      <x:c r="J10" s="8" t="str"/>
-      <x:c r="K10" s="8" t="str"/>
+      <x:c r="F10" s="8"/>
+      <x:c r="G10" s="8"/>
+      <x:c r="H10" s="8"/>
+      <x:c r="I10" s="8"/>
+      <x:c r="J10" s="8"/>
+      <x:c r="K10" s="8"/>
       <x:c r="L10" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M10" s="8" t="str"/>
+      <x:c r="M10" s="8"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="8" t="str">
@@ -574,16 +574,16 @@
       <x:c r="E11" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F11" s="8" t="str"/>
-      <x:c r="G11" s="8" t="str"/>
-      <x:c r="H11" s="8" t="str"/>
-      <x:c r="I11" s="8" t="str"/>
-      <x:c r="J11" s="8" t="str"/>
-      <x:c r="K11" s="8" t="str"/>
+      <x:c r="F11" s="8"/>
+      <x:c r="G11" s="8"/>
+      <x:c r="H11" s="8"/>
+      <x:c r="I11" s="8"/>
+      <x:c r="J11" s="8"/>
+      <x:c r="K11" s="8"/>
       <x:c r="L11" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M11" s="8" t="str"/>
+      <x:c r="M11" s="8"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="8" t="str">
@@ -601,16 +601,16 @@
       <x:c r="E12" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F12" s="8" t="str"/>
-      <x:c r="G12" s="8" t="str"/>
-      <x:c r="H12" s="8" t="str"/>
-      <x:c r="I12" s="8" t="str"/>
-      <x:c r="J12" s="8" t="str"/>
-      <x:c r="K12" s="8" t="str"/>
+      <x:c r="F12" s="8"/>
+      <x:c r="G12" s="8"/>
+      <x:c r="H12" s="8"/>
+      <x:c r="I12" s="8"/>
+      <x:c r="J12" s="8"/>
+      <x:c r="K12" s="8"/>
       <x:c r="L12" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M12" s="8" t="str"/>
+      <x:c r="M12" s="8"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="8" t="str">
@@ -628,16 +628,16 @@
       <x:c r="E13" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F13" s="8" t="str"/>
-      <x:c r="G13" s="8" t="str"/>
-      <x:c r="H13" s="8" t="str"/>
-      <x:c r="I13" s="8" t="str"/>
-      <x:c r="J13" s="8" t="str"/>
-      <x:c r="K13" s="8" t="str"/>
+      <x:c r="F13" s="8"/>
+      <x:c r="G13" s="8"/>
+      <x:c r="H13" s="8"/>
+      <x:c r="I13" s="8"/>
+      <x:c r="J13" s="8"/>
+      <x:c r="K13" s="8"/>
       <x:c r="L13" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M13" s="8" t="str"/>
+      <x:c r="M13" s="8"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
@@ -655,16 +655,16 @@
       <x:c r="E14" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F14" s="8" t="str"/>
-      <x:c r="G14" s="8" t="str"/>
-      <x:c r="H14" s="8" t="str"/>
-      <x:c r="I14" s="8" t="str"/>
-      <x:c r="J14" s="8" t="str"/>
-      <x:c r="K14" s="8" t="str"/>
+      <x:c r="F14" s="8"/>
+      <x:c r="G14" s="8"/>
+      <x:c r="H14" s="8"/>
+      <x:c r="I14" s="8"/>
+      <x:c r="J14" s="8"/>
+      <x:c r="K14" s="8"/>
       <x:c r="L14" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M14" s="8" t="str"/>
+      <x:c r="M14" s="8"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="8" t="str">
@@ -682,16 +682,16 @@
       <x:c r="E15" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F15" s="8" t="str"/>
-      <x:c r="G15" s="8" t="str"/>
-      <x:c r="H15" s="8" t="str"/>
-      <x:c r="I15" s="8" t="str"/>
-      <x:c r="J15" s="8" t="str"/>
-      <x:c r="K15" s="8" t="str"/>
+      <x:c r="F15" s="8"/>
+      <x:c r="G15" s="8"/>
+      <x:c r="H15" s="8"/>
+      <x:c r="I15" s="8"/>
+      <x:c r="J15" s="8"/>
+      <x:c r="K15" s="8"/>
       <x:c r="L15" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M15" s="8" t="str"/>
+      <x:c r="M15" s="8"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="8" t="str">
@@ -709,16 +709,16 @@
       <x:c r="E16" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F16" s="8" t="str"/>
-      <x:c r="G16" s="8" t="str"/>
-      <x:c r="H16" s="8" t="str"/>
-      <x:c r="I16" s="8" t="str"/>
-      <x:c r="J16" s="8" t="str"/>
-      <x:c r="K16" s="8" t="str"/>
+      <x:c r="F16" s="8"/>
+      <x:c r="G16" s="8"/>
+      <x:c r="H16" s="8"/>
+      <x:c r="I16" s="8"/>
+      <x:c r="J16" s="8"/>
+      <x:c r="K16" s="8"/>
       <x:c r="L16" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M16" s="8" t="str"/>
+      <x:c r="M16" s="8"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="8" t="str">
@@ -736,16 +736,16 @@
       <x:c r="E17" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F17" s="8" t="str"/>
-      <x:c r="G17" s="8" t="str"/>
-      <x:c r="H17" s="8" t="str"/>
-      <x:c r="I17" s="8" t="str"/>
-      <x:c r="J17" s="8" t="str"/>
-      <x:c r="K17" s="8" t="str"/>
+      <x:c r="F17" s="8"/>
+      <x:c r="G17" s="8"/>
+      <x:c r="H17" s="8"/>
+      <x:c r="I17" s="8"/>
+      <x:c r="J17" s="8"/>
+      <x:c r="K17" s="8"/>
       <x:c r="L17" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M17" s="8" t="str"/>
+      <x:c r="M17" s="8"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="8" t="str">
@@ -763,16 +763,16 @@
       <x:c r="E18" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F18" s="8" t="str"/>
-      <x:c r="G18" s="8" t="str"/>
-      <x:c r="H18" s="8" t="str"/>
-      <x:c r="I18" s="8" t="str"/>
-      <x:c r="J18" s="8" t="str"/>
-      <x:c r="K18" s="8" t="str"/>
+      <x:c r="F18" s="8"/>
+      <x:c r="G18" s="8"/>
+      <x:c r="H18" s="8"/>
+      <x:c r="I18" s="8"/>
+      <x:c r="J18" s="8"/>
+      <x:c r="K18" s="8"/>
       <x:c r="L18" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M18" s="8" t="str"/>
+      <x:c r="M18" s="8"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="8" t="str">
@@ -790,33 +790,33 @@
       <x:c r="E19" s="8" t="str">
         <x:v>hidden-answer</x:v>
       </x:c>
-      <x:c r="F19" s="8" t="str"/>
-      <x:c r="G19" s="8" t="str"/>
-      <x:c r="H19" s="8" t="str"/>
-      <x:c r="I19" s="8" t="str"/>
-      <x:c r="J19" s="8" t="str"/>
-      <x:c r="K19" s="8" t="str"/>
+      <x:c r="F19" s="8"/>
+      <x:c r="G19" s="8"/>
+      <x:c r="H19" s="8"/>
+      <x:c r="I19" s="8"/>
+      <x:c r="J19" s="8"/>
+      <x:c r="K19" s="8"/>
       <x:c r="L19" s="8" t="str">
         <x:v>yes</x:v>
       </x:c>
-      <x:c r="M19" s="8" t="str"/>
+      <x:c r="M19" s="8"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="8" t="str">
         <x:v>end_group</x:v>
       </x:c>
-      <x:c r="B20" s="8" t="str"/>
-      <x:c r="C20" s="8" t="str"/>
-      <x:c r="D20" s="8" t="str"/>
-      <x:c r="E20" s="8" t="str"/>
-      <x:c r="F20" s="8" t="str"/>
-      <x:c r="G20" s="8" t="str"/>
-      <x:c r="H20" s="8" t="str"/>
-      <x:c r="I20" s="8" t="str"/>
-      <x:c r="J20" s="8" t="str"/>
-      <x:c r="K20" s="8" t="str"/>
-      <x:c r="L20" s="8" t="str"/>
-      <x:c r="M20" s="8" t="str"/>
+      <x:c r="B20" s="8"/>
+      <x:c r="C20" s="8"/>
+      <x:c r="D20" s="8"/>
+      <x:c r="E20" s="8"/>
+      <x:c r="F20" s="8"/>
+      <x:c r="G20" s="8"/>
+      <x:c r="H20" s="8"/>
+      <x:c r="I20" s="8"/>
+      <x:c r="J20" s="8"/>
+      <x:c r="K20" s="8"/>
+      <x:c r="L20" s="8"/>
+      <x:c r="M20" s="8"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="8" t="str">
@@ -831,15 +831,204 @@
       <x:c r="D21" s="8" t="str">
         <x:v>Only fields relevant to this capability are stored, plus the shared FULL envelope.</x:v>
       </x:c>
-      <x:c r="E21" s="8" t="str"/>
-      <x:c r="F21" s="8" t="str"/>
-      <x:c r="G21" s="8" t="str"/>
-      <x:c r="H21" s="8" t="str"/>
-      <x:c r="I21" s="8" t="str"/>
-      <x:c r="J21" s="8" t="str"/>
-      <x:c r="K21" s="8" t="str"/>
-      <x:c r="L21" s="8" t="str"/>
-      <x:c r="M21" s="8" t="str"/>
+      <x:c r="E21" s="8"/>
+      <x:c r="F21" s="8"/>
+      <x:c r="G21" s="8"/>
+      <x:c r="H21" s="8"/>
+      <x:c r="I21" s="8"/>
+      <x:c r="J21" s="8"/>
+      <x:c r="K21" s="8"/>
+      <x:c r="L21" s="8"/>
+      <x:c r="M21" s="8"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>document_scan_timestamp_status</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Timestamp proof status</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>disabled, succeeded, or failed.</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F22" t="str"/>
+      <x:c r="G22" t="str"/>
+      <x:c r="H22" t="str"/>
+      <x:c r="I22" t="str"/>
+      <x:c r="J22" t="str"/>
+      <x:c r="K22" t="str"/>
+      <x:c r="L22" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M22" t="str"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>document_scan_timestamp_proof_uri</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Timestamp proof ZIP URI</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Returned when a TSA proof was created.</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F23" t="str"/>
+      <x:c r="G23" t="str"/>
+      <x:c r="H23" t="str"/>
+      <x:c r="I23" t="str"/>
+      <x:c r="J23" t="str"/>
+      <x:c r="K23" t="str"/>
+      <x:c r="L23" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M23" t="str"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>document_scan_timestamp_proof_filename</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Timestamp proof filename</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F24" t="str"/>
+      <x:c r="G24" t="str"/>
+      <x:c r="H24" t="str"/>
+      <x:c r="I24" t="str"/>
+      <x:c r="J24" t="str"/>
+      <x:c r="K24" t="str"/>
+      <x:c r="L24" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M24" t="str"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>document_scan_timestamp_authority</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Timestamp authority</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F25" t="str"/>
+      <x:c r="G25" t="str"/>
+      <x:c r="H25" t="str"/>
+      <x:c r="I25" t="str"/>
+      <x:c r="J25" t="str"/>
+      <x:c r="K25" t="str"/>
+      <x:c r="L25" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M25" t="str"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>document_scan_timestamp_time_iso</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Timestamp time</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Returned by MethodMesh.</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F26" t="str"/>
+      <x:c r="G26" t="str"/>
+      <x:c r="H26" t="str"/>
+      <x:c r="I26" t="str"/>
+      <x:c r="J26" t="str"/>
+      <x:c r="K26" t="str"/>
+      <x:c r="L26" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M26" t="str"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>document_scan_timestamp_sha256</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Timestamped PDF SHA-256</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Digest of the exact PDF covered by the proof.</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F27" t="str"/>
+      <x:c r="G27" t="str"/>
+      <x:c r="H27" t="str"/>
+      <x:c r="I27" t="str"/>
+      <x:c r="J27" t="str"/>
+      <x:c r="K27" t="str"/>
+      <x:c r="L27" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M27" t="str"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>text</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>document_scan_timestamp_error</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>Timestamp proof error</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>Returned when timestamp proof creation fails.</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>hidden-answer</x:v>
+      </x:c>
+      <x:c r="F28" t="str"/>
+      <x:c r="G28" t="str"/>
+      <x:c r="H28" t="str"/>
+      <x:c r="I28" t="str"/>
+      <x:c r="J28" t="str"/>
+      <x:c r="K28" t="str"/>
+      <x:c r="L28" t="str">
+        <x:v>yes</x:v>
+      </x:c>
+      <x:c r="M28" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>